<commit_message>
Mise à jour DLV/Prix KIBO4
</commit_message>
<xml_diff>
--- a/KIBO4/dlv-prix.xlsx
+++ b/KIBO4/dlv-prix.xlsx
@@ -13,9 +13,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="13">
-  <si>
-    <t>Date de mise à jour : 20/10/2026 00:50</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="22">
+  <si>
+    <t>Date de mise à jour : 20/10/2026 00:58</t>
   </si>
   <si>
     <t>Code Barre</t>
@@ -39,6 +39,39 @@
     <t>Dlv</t>
   </si>
   <si>
+    <t>3222472635604</t>
+  </si>
+  <si>
+    <t>50043027</t>
+  </si>
+  <si>
+    <t>SCE CRUDITE F HERBE 500ML CO NRK</t>
+  </si>
+  <si>
+    <t>500</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>01/10/2026</t>
+  </si>
+  <si>
+    <t>3165351111922</t>
+  </si>
+  <si>
+    <t>50043029</t>
+  </si>
+  <si>
+    <t>VINAIGRE BALSAMIQUE 500ML MILA FOOD</t>
+  </si>
+  <si>
+    <t>01/09/2026</t>
+  </si>
+  <si>
     <t>3222472434610</t>
   </si>
   <si>
@@ -46,12 +79,6 @@
   </si>
   <si>
     <t>SCE CRUDITE NATURE 500ML CO NRK</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>1</t>
   </si>
 </sst>
 </file>
@@ -467,7 +494,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -527,13 +554,59 @@
         <v>11</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="3" t="s">
-        <v>11</v>
+      <c r="E4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>